<commit_message>
Add HDLBits Attempt 2 progress and review materials
</commit_message>
<xml_diff>
--- a/HDLBits Attempt 1/HDLBits_Revision_Tracker.xlsx
+++ b/HDLBits Attempt 1/HDLBits_Revision_Tracker.xlsx
@@ -589,9 +589,9 @@
       <x:c r="B8" s="46" t="n">
         <x:v>46223</x:v>
       </x:c>
-      <x:c r="C8" s="31" t="e">
+      <x:c r="C8" s="31" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/always_case2","Priority encoder (always_case2)")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://hdlbits.01xz.net/wiki/always_case2, friendlyName=Priority encoder (always_case2)</x:v>
+        <x:v>Priority encoder (always_case2)</x:v>
       </x:c>
       <x:c r="D8" s="28" t="str">
         <x:v>Procedural logic · priority</x:v>
@@ -613,9 +613,9 @@
       <x:c r="B9" s="47" t="n">
         <x:v>46223</x:v>
       </x:c>
-      <x:c r="C9" s="32" t="e">
+      <x:c r="C9" s="32" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/adder100i","100-bit binary adder 2 (adder100i)")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://hdlbits.01xz.net/wiki/adder100i, friendlyName=100-bit binary adder 2 (adder100i)</x:v>
+        <x:v>100-bit binary adder 2 (adder100i)</x:v>
       </x:c>
       <x:c r="D9" s="29" t="str">
         <x:v>Generate loop · ripple-carry adder</x:v>
@@ -637,9 +637,9 @@
       <x:c r="B10" s="47" t="n">
         <x:v>46223</x:v>
       </x:c>
-      <x:c r="C10" s="32" t="e">
+      <x:c r="C10" s="32" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/sim/circuit8","Sequential circuit 8 (sim/circuit8)")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://hdlbits.01xz.net/wiki/sim/circuit8, friendlyName=Sequential circuit 8 (sim/circuit8)</x:v>
+        <x:v>Sequential circuit 8 (sim/circuit8)</x:v>
       </x:c>
       <x:c r="D10" s="29" t="str">
         <x:v>Waveform reading · sequential logic</x:v>
@@ -661,9 +661,9 @@
       <x:c r="B11" s="48" t="n">
         <x:v>46223</x:v>
       </x:c>
-      <x:c r="C11" s="33" t="e">
+      <x:c r="C11" s="33" t="str">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/lemmings2","Lemmings 2 (lemmings2)")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://hdlbits.01xz.net/wiki/lemmings2, friendlyName=Lemmings 2 (lemmings2)</x:v>
+        <x:v>Lemmings 2 (lemmings2)</x:v>
       </x:c>
       <x:c r="D11" s="30" t="str">
         <x:v>FSM · remembered direction</x:v>

</xml_diff>